<commit_message>
Stage 8.15B: temporarily withdraw PassControl from production
Stage 8.15B: temporarily withdraw PassControl from production
</commit_message>
<xml_diff>
--- a/ContentSource/PlayerContent/FMCodex_Canonical_Player_Content.xlsx
+++ b/ContentSource/PlayerContent/FMCodex_Canonical_Player_Content.xlsx
@@ -1442,37 +1442,29 @@
       <c r="V10" s="7" t="n"/>
       <c r="W10" s="7" t="inlineStr">
         <is>
-          <t>PassControl</t>
+          <t>ThroughBall</t>
         </is>
       </c>
       <c r="X10" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y10" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Y10" s="6" t="n">
-        <v>8</v>
-      </c>
       <c r="Z10" s="7" t="inlineStr">
         <is>
-          <t>ThroughBall</t>
+          <t>LongShot</t>
         </is>
       </c>
       <c r="AA10" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AB10" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC10" s="7" t="inlineStr">
-        <is>
-          <t>LongShot</t>
-        </is>
-      </c>
-      <c r="AD10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE10" s="6" t="n">
-        <v>5</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="AC10" s="7" t="n"/>
+      <c r="AD10" s="6" t="n"/>
+      <c r="AE10" s="6" t="n"/>
       <c r="AF10" s="8" t="inlineStr">
         <is>
           <t>前场组织核心；PassControl、ThroughBall与LongShot形成完整链路。</t>
@@ -1716,14 +1708,14 @@
       <c r="V13" s="10" t="n"/>
       <c r="W13" s="10" t="inlineStr">
         <is>
-          <t>PassControl</t>
+          <t>ThroughBall</t>
         </is>
       </c>
       <c r="X13" s="9" t="n">
         <v>7</v>
       </c>
       <c r="Y13" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Z13" s="10" t="n"/>
       <c r="AA13" s="10" t="n"/>
@@ -1802,37 +1794,29 @@
       <c r="V14" s="7" t="n"/>
       <c r="W14" s="7" t="inlineStr">
         <is>
-          <t>PassControl</t>
+          <t>ThroughBall</t>
         </is>
       </c>
       <c r="X14" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y14" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Y14" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="Z14" s="7" t="inlineStr">
         <is>
-          <t>ThroughBall</t>
+          <t>LongShot</t>
         </is>
       </c>
       <c r="AA14" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AB14" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC14" s="7" t="inlineStr">
-        <is>
-          <t>LongShot</t>
-        </is>
-      </c>
-      <c r="AD14" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE14" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="AC14" s="7" t="n"/>
+      <c r="AD14" s="6" t="n"/>
+      <c r="AE14" s="6" t="n"/>
       <c r="AF14" s="8" t="inlineStr">
         <is>
           <t>中场覆盖核心；高续航、推进和远射兼备。</t>
@@ -3052,26 +3036,18 @@
       <c r="V29" s="10" t="n"/>
       <c r="W29" s="10" t="inlineStr">
         <is>
-          <t>PassControl</t>
+          <t>ThroughBall</t>
         </is>
       </c>
       <c r="X29" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y29" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="Y29" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="Z29" s="10" t="inlineStr">
-        <is>
-          <t>ThroughBall</t>
-        </is>
-      </c>
-      <c r="AA29" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="AB29" s="9" t="n">
-        <v>6</v>
-      </c>
+      <c r="Z29" s="10" t="n"/>
+      <c r="AA29" s="9" t="n"/>
+      <c r="AB29" s="9" t="n"/>
       <c r="AC29" s="10" t="n"/>
       <c r="AD29" s="10" t="n"/>
       <c r="AE29" s="10" t="n"/>
@@ -3146,26 +3122,18 @@
       <c r="V30" s="7" t="n"/>
       <c r="W30" s="7" t="inlineStr">
         <is>
-          <t>PassControl</t>
+          <t>ThroughBall</t>
         </is>
       </c>
       <c r="X30" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y30" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="Y30" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Z30" s="7" t="inlineStr">
-        <is>
-          <t>ThroughBall</t>
-        </is>
-      </c>
-      <c r="AA30" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="AB30" s="6" t="n">
-        <v>6</v>
-      </c>
+      <c r="Z30" s="7" t="n"/>
+      <c r="AA30" s="6" t="n"/>
+      <c r="AB30" s="6" t="n"/>
       <c r="AC30" s="7" t="n"/>
       <c r="AD30" s="7" t="n"/>
       <c r="AE30" s="7" t="n"/>
@@ -3240,7 +3208,7 @@
       <c r="V31" s="10" t="n"/>
       <c r="W31" s="10" t="inlineStr">
         <is>
-          <t>PassControl</t>
+          <t>ThroughBall</t>
         </is>
       </c>
       <c r="X31" s="9" t="n">
@@ -3249,17 +3217,9 @@
       <c r="Y31" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="Z31" s="10" t="inlineStr">
-        <is>
-          <t>ThroughBall</t>
-        </is>
-      </c>
-      <c r="AA31" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB31" s="9" t="n">
-        <v>8</v>
-      </c>
+      <c r="Z31" s="10" t="n"/>
+      <c r="AA31" s="9" t="n"/>
+      <c r="AB31" s="9" t="n"/>
       <c r="AC31" s="10" t="n"/>
       <c r="AD31" s="10" t="n"/>
       <c r="AE31" s="10" t="n"/>
@@ -4209,7 +4169,7 @@
       </c>
       <c r="B3" s="19" t="inlineStr">
         <is>
-          <t>2026-09-27；schemaVersion 3；balanceContentVersion Prototype40_v1。</t>
+          <t>当前实验：schemaVersion 3；balanceContentVersion Prototype40_v2。2026-09-27，Stage 8.15B。</t>
         </is>
       </c>
     </row>
@@ -4300,12 +4260,12 @@
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>五战术基线</t>
+          <t>四战术实验</t>
         </is>
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>LongShot / CutInsideShot / PassControl / Cross / ThroughBall；本次恢复不退出 PassControl，不修改 Zubimendi。</t>
+          <t>Stage 8.15B 暂时退出 PassControl。生产保留 LongShot / CutInsideShot / Cross / ThroughBall；苏比门迪为 ThroughBall 7–8。</t>
         </is>
       </c>
     </row>

</xml_diff>